<commit_message>
fix(documentation): revision of initial documentation
</commit_message>
<xml_diff>
--- a/documentation/user_story_mapping/user_story_map.xlsx
+++ b/documentation/user_story_mapping/user_story_map.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/khelandesai/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_07D0BAD9517A949E621180974786FE39332BC243" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7C4D238-E5BE-0243-B1BF-F6F889E244F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="88">
   <si>
     <t>Consultation Scheduler — User Story Map</t>
   </si>
@@ -47,6 +47,30 @@
   </si>
   <si>
     <t>Enhancements</t>
+  </si>
+  <si>
+    <t>As a user, I want to register and log in with a role, so that I can access features relevant to me as a student or lecturer.</t>
+  </si>
+  <si>
+    <t>As a lecturer, I want to configure my availability and consultation preferences, so that students can only book sessions within my defined constraints.</t>
+  </si>
+  <si>
+    <t>As a student, I want to browse lecturers and their availability, so that I can find and choose who to book a consultation with.</t>
+  </si>
+  <si>
+    <t>As a student, I want to create and join consultations, so that I can arrange group meetings with a lecturer without clashing with existing bookings.</t>
+  </si>
+  <si>
+    <t>As a user, I want a role-specific dashboard showing upcoming consultations and their status, so that I can manage my schedule at a glance.</t>
+  </si>
+  <si>
+    <t>As a student or lecturer, I want to cancel a consultation, so that the slot is freed up and all affected parties are notified.</t>
+  </si>
+  <si>
+    <t>As an administrator, I want all user actions automatically logged and viewable, so that there is a complete audit trail of system activity.</t>
+  </si>
+  <si>
+    <t>As a user, I want additional features such as following lecturers, Google sign-in, and security improvements, so that the system is more convenient and trustworthy to use.</t>
   </si>
   <si>
     <t>User Registration &amp; Login</t>
@@ -198,89 +222,77 @@
     <t>As a user, I want to add my courses and degree to my profile so that I can search for other users in my courses.</t>
   </si>
   <si>
-    <t>Sprint 1</t>
+    <t>Developer Tasks</t>
   </si>
   <si>
     <t>↓ Sprint 1</t>
   </si>
   <si>
-    <t>Register</t>
-  </si>
-  <si>
-    <t>Select role</t>
-  </si>
-  <si>
-    <t>Navigate to dashboard</t>
-  </si>
-  <si>
-    <t>Set availability</t>
-  </si>
-  <si>
-    <t>Set consultation limits</t>
-  </si>
-  <si>
-    <t>Browse lecturers</t>
-  </si>
-  <si>
-    <t>Log in</t>
-  </si>
-  <si>
-    <t>Register with role</t>
-  </si>
-  <si>
-    <t>Access pages</t>
-  </si>
-  <si>
-    <t>View availability form</t>
-  </si>
-  <si>
-    <t>View settings form</t>
-  </si>
-  <si>
-    <t>View lecturer list</t>
-  </si>
-  <si>
-    <t>Validate credentials</t>
-  </si>
-  <si>
-    <t>Save availability</t>
-  </si>
-  <si>
-    <t>Save settings</t>
-  </si>
-  <si>
-    <t>View lecturer availability</t>
-  </si>
-  <si>
-    <t>View saved availability</t>
-  </si>
-  <si>
-    <t>Validate settings</t>
-  </si>
-  <si>
-    <t>Sprint 2</t>
+    <t>As a developer, I want to build a registration flow with input validation, so that new users can securely create an account.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to capture and store a user's role at sign-up, so that role-specific behaviour is available from first login.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to redirect users to a role-appropriate dashboard on login, so that each user lands on the correct view.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to build availability management for lecturers, so that they can set and update their weekly time slots.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to implement consultation preference settings, so that lecturer-defined constraints are enforced during booking.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to build a lecturer browsing screen with availability data, so that students can find and choose who to book with.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to tie role assignment to the registration process, so that permissions are applied from account creation.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to restrict page access based on user role, so that users can only reach views relevant to them.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to render the availability form pre-populated with saved data, so that lecturers can review and edit their schedule.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to render the consultation settings form with current config, so that lecturers can view and update their preferences.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to build a lecturer list view, so that students can browse all lecturers available for booking.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to validate login credentials and handle failures gracefully, so that only authorised users can access the system.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to persist availability data when a lecturer saves their schedule, so that it is stored and reflected across the app.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to save consultation settings to the database on submission, so that lecturer constraints are consistently applied.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to display a lecturer's availability on their profile, so that students can see when they are bookable.</t>
   </si>
   <si>
     <t>↓ Sprint 2</t>
   </si>
   <si>
-    <t>Sprint 3</t>
-  </si>
-  <si>
     <t>↓ Sprint 3</t>
   </si>
   <si>
-    <t>Sprint 4</t>
-  </si>
-  <si>
     <t>↓ Sprint 4</t>
+  </si>
+  <si>
+    <t>As a developer, I want to build a login flow with session management, so that authenticated users can access the system.</t>
+  </si>
+  <si>
+    <t>User Epics</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -355,6 +367,20 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="0"/>
+      <name val="Calibri (Body)"/>
     </font>
   </fonts>
   <fills count="17">
@@ -578,7 +604,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -623,48 +649,55 @@
     <xf numFmtId="0" fontId="7" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -967,328 +1000,334 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y24"/>
+  <dimension ref="A1:Y25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12" style="1" customWidth="1"/>
     <col min="2" max="25" width="22" style="1" customWidth="1"/>
-    <col min="26" max="26" width="8.83203125" style="1" customWidth="1"/>
-    <col min="27" max="16384" width="8.83203125" style="1"/>
+    <col min="26" max="27" width="8.83203125" style="1" customWidth="1"/>
+    <col min="28" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="22"/>
-      <c r="M1" s="22"/>
-      <c r="N1" s="22"/>
-      <c r="O1" s="22"/>
-      <c r="P1" s="22"/>
-      <c r="Q1" s="22"/>
-      <c r="R1" s="22"/>
-      <c r="S1" s="22"/>
-      <c r="T1" s="22"/>
-      <c r="U1" s="22"/>
-      <c r="V1" s="22"/>
-      <c r="W1" s="22"/>
-      <c r="X1" s="22"/>
-      <c r="Y1" s="22"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="21"/>
+      <c r="O1" s="21"/>
+      <c r="P1" s="21"/>
+      <c r="Q1" s="21"/>
+      <c r="R1" s="21"/>
+      <c r="S1" s="21"/>
+      <c r="T1" s="21"/>
+      <c r="U1" s="21"/>
+      <c r="V1" s="21"/>
+      <c r="W1" s="21"/>
+      <c r="X1" s="21"/>
+      <c r="Y1" s="21"/>
     </row>
     <row r="2" spans="1:25" s="11" customFormat="1" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="10"/>
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="28" t="s">
+      <c r="C2" s="23"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="29"/>
+      <c r="F2" s="24"/>
       <c r="G2" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="28" t="s">
+      <c r="H2" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="19"/>
-      <c r="L2" s="29"/>
-      <c r="M2" s="28" t="s">
+      <c r="I2" s="23"/>
+      <c r="J2" s="23"/>
+      <c r="K2" s="23"/>
+      <c r="L2" s="24"/>
+      <c r="M2" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="N2" s="19"/>
-      <c r="O2" s="19"/>
-      <c r="P2" s="29"/>
-      <c r="Q2" s="28" t="s">
+      <c r="N2" s="23"/>
+      <c r="O2" s="23"/>
+      <c r="P2" s="24"/>
+      <c r="Q2" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="R2" s="29"/>
-      <c r="S2" s="28" t="s">
+      <c r="R2" s="24"/>
+      <c r="S2" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="T2" s="29"/>
-      <c r="U2" s="34" t="s">
+      <c r="T2" s="24"/>
+      <c r="U2" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="V2" s="35"/>
-      <c r="W2" s="35"/>
-      <c r="X2" s="35"/>
-      <c r="Y2" s="35"/>
-    </row>
-    <row r="3" spans="1:25" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="2"/>
-      <c r="B3" s="3" t="s">
+      <c r="V2" s="31"/>
+      <c r="W2" s="31"/>
+      <c r="X2" s="31"/>
+      <c r="Y2" s="31"/>
+    </row>
+    <row r="3" spans="1:25" s="18" customFormat="1" ht="230" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="B3" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="23"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="F3" s="24"/>
+      <c r="G3" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="H3" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="I3" s="23"/>
+      <c r="J3" s="23"/>
+      <c r="K3" s="23"/>
+      <c r="L3" s="24"/>
+      <c r="M3" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="N3" s="23"/>
+      <c r="O3" s="23"/>
+      <c r="P3" s="24"/>
+      <c r="Q3" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="R3" s="24"/>
+      <c r="S3" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="T3" s="24"/>
+      <c r="U3" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="V3" s="23"/>
+      <c r="W3" s="23"/>
+      <c r="X3" s="23"/>
+      <c r="Y3" s="23"/>
+    </row>
+    <row r="4" spans="1:25" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="2"/>
+      <c r="B4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="M3" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="N3" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="O3" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="P3" s="3" t="s">
+      <c r="H4" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="Q3" s="3" t="s">
+      <c r="I4" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="R3" s="3" t="s">
+      <c r="J4" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="S3" s="3" t="s">
+      <c r="K4" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="T3" s="3" t="s">
+      <c r="L4" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="U3" s="3" t="s">
+      <c r="M4" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="V3" s="3" t="s">
+      <c r="N4" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="W3" s="3" t="s">
+      <c r="O4" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="X3" s="3" t="s">
+      <c r="P4" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="Y3" s="3" t="s">
+      <c r="Q4" s="3" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="4" spans="1:25" ht="136" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
+      <c r="R4" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="S4" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="T4" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="U4" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="V4" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="W4" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="X4" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="Y4" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="I4" s="5" t="s">
+    </row>
+    <row r="5" spans="1:25" ht="136" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="J4" s="5" t="s">
+      <c r="B5" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="K4" s="5" t="s">
+      <c r="C5" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="L4" s="5" t="s">
+      <c r="D5" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="M4" s="5" t="s">
+      <c r="E5" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="N4" s="5" t="s">
+      <c r="F5" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="O4" s="5" t="s">
+      <c r="G5" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="P4" s="5" t="s">
+      <c r="H5" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="Q4" s="5" t="s">
+      <c r="I5" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="R4" s="5" t="s">
+      <c r="J5" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="S4" s="5" t="s">
+      <c r="K5" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="T4" s="5" t="s">
+      <c r="L5" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="U4" s="5" t="s">
+      <c r="M5" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="V4" s="5" t="s">
+      <c r="N5" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="W4" s="5" t="s">
+      <c r="O5" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="X4" s="5" t="s">
+      <c r="P5" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="Y4" s="5" t="s">
+      <c r="Q5" s="5" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="5" spans="1:25" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="32" t="s">
+      <c r="R5" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="B5" s="26" t="s">
+      <c r="S5" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C5" s="19"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="19"/>
-      <c r="G5" s="19"/>
-      <c r="H5" s="19"/>
-      <c r="I5" s="19"/>
-      <c r="J5" s="19"/>
-      <c r="K5" s="19"/>
-      <c r="L5" s="19"/>
-      <c r="M5" s="19"/>
-      <c r="N5" s="19"/>
-      <c r="O5" s="19"/>
-      <c r="P5" s="19"/>
-      <c r="Q5" s="19"/>
-      <c r="R5" s="19"/>
-      <c r="S5" s="19"/>
-      <c r="T5" s="19"/>
-      <c r="U5" s="19"/>
-      <c r="V5" s="19"/>
-      <c r="W5" s="19"/>
-      <c r="X5" s="19"/>
-      <c r="Y5" s="19"/>
-    </row>
-    <row r="6" spans="1:25" ht="66" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="24"/>
-      <c r="B6" s="6" t="s">
+      <c r="T5" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="U5" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="V5" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="W5" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="X5" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="Y5" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6"/>
-      <c r="J6" s="6"/>
-      <c r="K6" s="6"/>
-      <c r="L6" s="6"/>
-      <c r="M6" s="6"/>
-      <c r="N6" s="13"/>
-      <c r="O6" s="6"/>
-      <c r="P6" s="6"/>
-      <c r="Q6" s="6"/>
-      <c r="R6" s="6"/>
-      <c r="S6" s="6"/>
-      <c r="T6" s="6"/>
-      <c r="U6" s="6"/>
-      <c r="V6" s="6"/>
-      <c r="W6" s="6"/>
-      <c r="X6" s="15"/>
-      <c r="Y6" s="15"/>
-    </row>
-    <row r="7" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="24"/>
+    </row>
+    <row r="6" spans="1:25" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="28" t="s">
+        <v>66</v>
+      </c>
+      <c r="B6" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="C6" s="23"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="23"/>
+      <c r="I6" s="23"/>
+      <c r="J6" s="23"/>
+      <c r="K6" s="23"/>
+      <c r="L6" s="23"/>
+      <c r="M6" s="23"/>
+      <c r="N6" s="23"/>
+      <c r="O6" s="23"/>
+      <c r="P6" s="23"/>
+      <c r="Q6" s="23"/>
+      <c r="R6" s="23"/>
+      <c r="S6" s="23"/>
+      <c r="T6" s="23"/>
+      <c r="U6" s="23"/>
+      <c r="V6" s="23"/>
+      <c r="W6" s="23"/>
+      <c r="X6" s="23"/>
+      <c r="Y6" s="23"/>
+    </row>
+    <row r="7" spans="1:25" ht="123" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="26"/>
       <c r="B7" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H7" s="6"/>
       <c r="I7" s="6"/>
@@ -1296,7 +1335,7 @@
       <c r="K7" s="6"/>
       <c r="L7" s="6"/>
       <c r="M7" s="6"/>
-      <c r="N7" s="14"/>
+      <c r="N7" s="13"/>
       <c r="O7" s="6"/>
       <c r="P7" s="6"/>
       <c r="Q7" s="6"/>
@@ -1306,24 +1345,28 @@
       <c r="U7" s="6"/>
       <c r="V7" s="6"/>
       <c r="W7" s="6"/>
-      <c r="X7" s="17"/>
-      <c r="Y7" s="16"/>
-    </row>
-    <row r="8" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="24"/>
+      <c r="X7" s="15"/>
+      <c r="Y7" s="15"/>
+    </row>
+    <row r="8" spans="1:25" ht="125" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="26"/>
       <c r="B8" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
+        <v>86</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>75</v>
+      </c>
       <c r="E8" s="6" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="H8" s="6"/>
       <c r="I8" s="6"/>
@@ -1331,7 +1374,7 @@
       <c r="K8" s="6"/>
       <c r="L8" s="6"/>
       <c r="M8" s="6"/>
-      <c r="N8" s="6"/>
+      <c r="N8" s="14"/>
       <c r="O8" s="6"/>
       <c r="P8" s="6"/>
       <c r="Q8" s="6"/>
@@ -1341,21 +1384,25 @@
       <c r="U8" s="6"/>
       <c r="V8" s="6"/>
       <c r="W8" s="6"/>
-      <c r="X8" s="6"/>
-      <c r="Y8" s="6"/>
-    </row>
-    <row r="9" spans="1:25" ht="78" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="25"/>
-      <c r="B9" s="6"/>
+      <c r="X8" s="17"/>
+      <c r="Y8" s="16"/>
+    </row>
+    <row r="9" spans="1:25" ht="120" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="26"/>
+      <c r="B9" s="6" t="s">
+        <v>79</v>
+      </c>
       <c r="C9" s="6"/>
       <c r="D9" s="6"/>
       <c r="E9" s="6" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="G9" s="6"/>
+        <v>81</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>82</v>
+      </c>
       <c r="H9" s="6"/>
       <c r="I9" s="6"/>
       <c r="J9" s="6"/>
@@ -1375,66 +1422,66 @@
       <c r="X9" s="6"/>
       <c r="Y9" s="6"/>
     </row>
-    <row r="10" spans="1:25" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="23" t="s">
-        <v>78</v>
-      </c>
-      <c r="B10" s="20" t="s">
-        <v>79</v>
-      </c>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
-      <c r="G10" s="19"/>
-      <c r="H10" s="19"/>
-      <c r="I10" s="19"/>
-      <c r="J10" s="19"/>
-      <c r="K10" s="19"/>
-      <c r="L10" s="19"/>
-      <c r="M10" s="19"/>
-      <c r="N10" s="19"/>
-      <c r="O10" s="19"/>
-      <c r="P10" s="19"/>
-      <c r="Q10" s="19"/>
-      <c r="R10" s="19"/>
-      <c r="S10" s="19"/>
-      <c r="T10" s="19"/>
-      <c r="U10" s="19"/>
-      <c r="V10" s="19"/>
-      <c r="W10" s="19"/>
-      <c r="X10" s="19"/>
-      <c r="Y10" s="19"/>
-    </row>
-    <row r="11" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="24"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
-      <c r="H11" s="7"/>
-      <c r="I11" s="7"/>
-      <c r="J11" s="7"/>
-      <c r="K11" s="7"/>
-      <c r="L11" s="7"/>
-      <c r="M11" s="7"/>
-      <c r="N11" s="7"/>
-      <c r="O11" s="7"/>
-      <c r="P11" s="7"/>
-      <c r="Q11" s="7"/>
-      <c r="R11" s="7"/>
-      <c r="S11" s="7"/>
-      <c r="T11" s="7"/>
-      <c r="U11" s="7"/>
-      <c r="V11" s="7"/>
-      <c r="W11" s="7"/>
-      <c r="X11" s="7"/>
-      <c r="Y11" s="7"/>
+    <row r="10" spans="1:25" ht="78" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="27"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="6"/>
+      <c r="K10" s="6"/>
+      <c r="L10" s="6"/>
+      <c r="M10" s="6"/>
+      <c r="N10" s="6"/>
+      <c r="O10" s="6"/>
+      <c r="P10" s="6"/>
+      <c r="Q10" s="6"/>
+      <c r="R10" s="6"/>
+      <c r="S10" s="6"/>
+      <c r="T10" s="6"/>
+      <c r="U10" s="6"/>
+      <c r="V10" s="6"/>
+      <c r="W10" s="6"/>
+      <c r="X10" s="6"/>
+      <c r="Y10" s="6"/>
+    </row>
+    <row r="11" spans="1:25" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" s="36" t="s">
+        <v>83</v>
+      </c>
+      <c r="C11" s="23"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="23"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="23"/>
+      <c r="J11" s="23"/>
+      <c r="K11" s="23"/>
+      <c r="L11" s="23"/>
+      <c r="M11" s="23"/>
+      <c r="N11" s="23"/>
+      <c r="O11" s="23"/>
+      <c r="P11" s="23"/>
+      <c r="Q11" s="23"/>
+      <c r="R11" s="23"/>
+      <c r="S11" s="23"/>
+      <c r="T11" s="23"/>
+      <c r="U11" s="23"/>
+      <c r="V11" s="23"/>
+      <c r="W11" s="23"/>
+      <c r="X11" s="23"/>
+      <c r="Y11" s="23"/>
     </row>
     <row r="12" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="24"/>
+      <c r="A12" s="26"/>
       <c r="B12" s="7"/>
       <c r="C12" s="7"/>
       <c r="D12" s="7"/>
@@ -1461,7 +1508,7 @@
       <c r="Y12" s="7"/>
     </row>
     <row r="13" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="24"/>
+      <c r="A13" s="26"/>
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
@@ -1488,7 +1535,7 @@
       <c r="Y13" s="7"/>
     </row>
     <row r="14" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="25"/>
+      <c r="A14" s="26"/>
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
       <c r="D14" s="7"/>
@@ -1514,66 +1561,66 @@
       <c r="X14" s="7"/>
       <c r="Y14" s="7"/>
     </row>
-    <row r="15" spans="1:25" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="33" t="s">
-        <v>80</v>
-      </c>
-      <c r="B15" s="31" t="s">
-        <v>81</v>
-      </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
-      <c r="G15" s="19"/>
-      <c r="H15" s="19"/>
-      <c r="I15" s="19"/>
-      <c r="J15" s="19"/>
-      <c r="K15" s="19"/>
-      <c r="L15" s="19"/>
-      <c r="M15" s="19"/>
-      <c r="N15" s="19"/>
-      <c r="O15" s="19"/>
-      <c r="P15" s="19"/>
-      <c r="Q15" s="19"/>
-      <c r="R15" s="19"/>
-      <c r="S15" s="19"/>
-      <c r="T15" s="19"/>
-      <c r="U15" s="19"/>
-      <c r="V15" s="19"/>
-      <c r="W15" s="19"/>
-      <c r="X15" s="19"/>
-      <c r="Y15" s="19"/>
-    </row>
-    <row r="16" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="24"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
-      <c r="J16" s="8"/>
-      <c r="K16" s="8"/>
-      <c r="L16" s="8"/>
-      <c r="M16" s="8"/>
-      <c r="N16" s="8"/>
-      <c r="O16" s="8"/>
-      <c r="P16" s="8"/>
-      <c r="Q16" s="8"/>
-      <c r="R16" s="8"/>
-      <c r="S16" s="8"/>
-      <c r="T16" s="8"/>
-      <c r="U16" s="8"/>
-      <c r="V16" s="8"/>
-      <c r="W16" s="8"/>
-      <c r="X16" s="8"/>
-      <c r="Y16" s="8"/>
+    <row r="15" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="27"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="7"/>
+      <c r="J15" s="7"/>
+      <c r="K15" s="7"/>
+      <c r="L15" s="7"/>
+      <c r="M15" s="7"/>
+      <c r="N15" s="7"/>
+      <c r="O15" s="7"/>
+      <c r="P15" s="7"/>
+      <c r="Q15" s="7"/>
+      <c r="R15" s="7"/>
+      <c r="S15" s="7"/>
+      <c r="T15" s="7"/>
+      <c r="U15" s="7"/>
+      <c r="V15" s="7"/>
+      <c r="W15" s="7"/>
+      <c r="X15" s="7"/>
+      <c r="Y15" s="7"/>
+    </row>
+    <row r="16" spans="1:25" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="38" t="s">
+        <v>66</v>
+      </c>
+      <c r="B16" s="37" t="s">
+        <v>84</v>
+      </c>
+      <c r="C16" s="23"/>
+      <c r="D16" s="23"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="23"/>
+      <c r="G16" s="23"/>
+      <c r="H16" s="23"/>
+      <c r="I16" s="23"/>
+      <c r="J16" s="23"/>
+      <c r="K16" s="23"/>
+      <c r="L16" s="23"/>
+      <c r="M16" s="23"/>
+      <c r="N16" s="23"/>
+      <c r="O16" s="23"/>
+      <c r="P16" s="23"/>
+      <c r="Q16" s="23"/>
+      <c r="R16" s="23"/>
+      <c r="S16" s="23"/>
+      <c r="T16" s="23"/>
+      <c r="U16" s="23"/>
+      <c r="V16" s="23"/>
+      <c r="W16" s="23"/>
+      <c r="X16" s="23"/>
+      <c r="Y16" s="23"/>
     </row>
     <row r="17" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="24"/>
+      <c r="A17" s="26"/>
       <c r="B17" s="8"/>
       <c r="C17" s="8"/>
       <c r="D17" s="8"/>
@@ -1600,7 +1647,7 @@
       <c r="Y17" s="8"/>
     </row>
     <row r="18" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="24"/>
+      <c r="A18" s="26"/>
       <c r="B18" s="8"/>
       <c r="C18" s="8"/>
       <c r="D18" s="8"/>
@@ -1627,7 +1674,7 @@
       <c r="Y18" s="8"/>
     </row>
     <row r="19" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="25"/>
+      <c r="A19" s="26"/>
       <c r="B19" s="8"/>
       <c r="C19" s="8"/>
       <c r="D19" s="8"/>
@@ -1653,66 +1700,66 @@
       <c r="X19" s="8"/>
       <c r="Y19" s="8"/>
     </row>
-    <row r="20" spans="1:25" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="27" t="s">
-        <v>82</v>
-      </c>
-      <c r="B20" s="18" t="s">
-        <v>83</v>
-      </c>
-      <c r="C20" s="19"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="19"/>
-      <c r="F20" s="19"/>
-      <c r="G20" s="19"/>
-      <c r="H20" s="19"/>
-      <c r="I20" s="19"/>
-      <c r="J20" s="19"/>
-      <c r="K20" s="19"/>
-      <c r="L20" s="19"/>
-      <c r="M20" s="19"/>
-      <c r="N20" s="19"/>
-      <c r="O20" s="19"/>
-      <c r="P20" s="19"/>
-      <c r="Q20" s="19"/>
-      <c r="R20" s="19"/>
-      <c r="S20" s="19"/>
-      <c r="T20" s="19"/>
-      <c r="U20" s="19"/>
-      <c r="V20" s="19"/>
-      <c r="W20" s="19"/>
-      <c r="X20" s="19"/>
-      <c r="Y20" s="19"/>
-    </row>
-    <row r="21" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="24"/>
-      <c r="B21" s="9"/>
-      <c r="C21" s="9"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
-      <c r="G21" s="9"/>
-      <c r="H21" s="9"/>
-      <c r="I21" s="9"/>
-      <c r="J21" s="9"/>
-      <c r="K21" s="9"/>
-      <c r="L21" s="9"/>
-      <c r="M21" s="9"/>
-      <c r="N21" s="9"/>
-      <c r="O21" s="9"/>
-      <c r="P21" s="9"/>
-      <c r="Q21" s="9"/>
-      <c r="R21" s="9"/>
-      <c r="S21" s="9"/>
-      <c r="T21" s="9"/>
-      <c r="U21" s="9"/>
-      <c r="V21" s="9"/>
-      <c r="W21" s="9"/>
-      <c r="X21" s="9"/>
-      <c r="Y21" s="9"/>
+    <row r="20" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="27"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
+      <c r="I20" s="8"/>
+      <c r="J20" s="8"/>
+      <c r="K20" s="8"/>
+      <c r="L20" s="8"/>
+      <c r="M20" s="8"/>
+      <c r="N20" s="8"/>
+      <c r="O20" s="8"/>
+      <c r="P20" s="8"/>
+      <c r="Q20" s="8"/>
+      <c r="R20" s="8"/>
+      <c r="S20" s="8"/>
+      <c r="T20" s="8"/>
+      <c r="U20" s="8"/>
+      <c r="V20" s="8"/>
+      <c r="W20" s="8"/>
+      <c r="X20" s="8"/>
+      <c r="Y20" s="8"/>
+    </row>
+    <row r="21" spans="1:25" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="35" t="s">
+        <v>66</v>
+      </c>
+      <c r="B21" s="34" t="s">
+        <v>85</v>
+      </c>
+      <c r="C21" s="23"/>
+      <c r="D21" s="23"/>
+      <c r="E21" s="23"/>
+      <c r="F21" s="23"/>
+      <c r="G21" s="23"/>
+      <c r="H21" s="23"/>
+      <c r="I21" s="23"/>
+      <c r="J21" s="23"/>
+      <c r="K21" s="23"/>
+      <c r="L21" s="23"/>
+      <c r="M21" s="23"/>
+      <c r="N21" s="23"/>
+      <c r="O21" s="23"/>
+      <c r="P21" s="23"/>
+      <c r="Q21" s="23"/>
+      <c r="R21" s="23"/>
+      <c r="S21" s="23"/>
+      <c r="T21" s="23"/>
+      <c r="U21" s="23"/>
+      <c r="V21" s="23"/>
+      <c r="W21" s="23"/>
+      <c r="X21" s="23"/>
+      <c r="Y21" s="23"/>
     </row>
     <row r="22" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="24"/>
+      <c r="A22" s="26"/>
       <c r="B22" s="9"/>
       <c r="C22" s="9"/>
       <c r="D22" s="9"/>
@@ -1739,7 +1786,7 @@
       <c r="Y22" s="9"/>
     </row>
     <row r="23" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="24"/>
+      <c r="A23" s="26"/>
       <c r="B23" s="9"/>
       <c r="C23" s="9"/>
       <c r="D23" s="9"/>
@@ -1766,7 +1813,7 @@
       <c r="Y23" s="9"/>
     </row>
     <row r="24" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="25"/>
+      <c r="A24" s="26"/>
       <c r="B24" s="9"/>
       <c r="C24" s="9"/>
       <c r="D24" s="9"/>
@@ -1792,24 +1839,58 @@
       <c r="X24" s="9"/>
       <c r="Y24" s="9"/>
     </row>
+    <row r="25" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="27"/>
+      <c r="B25" s="9"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="9"/>
+      <c r="I25" s="9"/>
+      <c r="J25" s="9"/>
+      <c r="K25" s="9"/>
+      <c r="L25" s="9"/>
+      <c r="M25" s="9"/>
+      <c r="N25" s="9"/>
+      <c r="O25" s="9"/>
+      <c r="P25" s="9"/>
+      <c r="Q25" s="9"/>
+      <c r="R25" s="9"/>
+      <c r="S25" s="9"/>
+      <c r="T25" s="9"/>
+      <c r="U25" s="9"/>
+      <c r="V25" s="9"/>
+      <c r="W25" s="9"/>
+      <c r="X25" s="9"/>
+      <c r="Y25" s="9"/>
+    </row>
   </sheetData>
-  <mergeCells count="16">
-    <mergeCell ref="B20:Y20"/>
-    <mergeCell ref="B10:Y10"/>
+  <mergeCells count="23">
+    <mergeCell ref="B21:Y21"/>
+    <mergeCell ref="A21:A25"/>
+    <mergeCell ref="Q3:R3"/>
+    <mergeCell ref="M3:P3"/>
+    <mergeCell ref="B11:Y11"/>
+    <mergeCell ref="S3:T3"/>
+    <mergeCell ref="B16:Y16"/>
+    <mergeCell ref="A16:A20"/>
     <mergeCell ref="A1:Y1"/>
-    <mergeCell ref="A10:A14"/>
-    <mergeCell ref="B5:Y5"/>
-    <mergeCell ref="A20:A24"/>
     <mergeCell ref="M2:P2"/>
+    <mergeCell ref="A11:A15"/>
+    <mergeCell ref="A6:A10"/>
+    <mergeCell ref="H3:L3"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="Q2:R2"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="S2:T2"/>
+    <mergeCell ref="U2:Y2"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="H2:L2"/>
-    <mergeCell ref="S2:T2"/>
-    <mergeCell ref="Q2:R2"/>
-    <mergeCell ref="B15:Y15"/>
-    <mergeCell ref="A5:A9"/>
-    <mergeCell ref="A15:A19"/>
+    <mergeCell ref="B6:Y6"/>
     <mergeCell ref="E2:F2"/>
-    <mergeCell ref="U2:Y2"/>
+    <mergeCell ref="U3:Y3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(documentation): add sprint retrospective and update user story map
</commit_message>
<xml_diff>
--- a/documentation/user_story_mapping/user_story_map.xlsx
+++ b/documentation/user_story_mapping/user_story_map.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/khelandesai/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\khela\ELEN4010 Group Lab\2026-group-lab-001\documentation\user_story_mapping\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7C4D238-E5BE-0243-B1BF-F6F889E244F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E24A244B-9F51-4F49-8C37-61DA4A67C6E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Story Map" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="99">
   <si>
     <t>Consultation Scheduler — User Story Map</t>
   </si>
@@ -286,13 +286,46 @@
   </si>
   <si>
     <t>User Epics</t>
+  </si>
+  <si>
+    <t>As a developer, I want to build the consultation creation form and POST route, so that a student can submit a new booking.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to implement an overlap detection service, so that no two consultations for the same lecturer occupy the same time slot.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to build a POST /consultations/:id/join endpoint, so that a student can add themselves to an existing consultation.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to enforce the max consultations per day limit at booking time, so that the lecturer is not overbooked on any given day.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to add query-parameter filtering to the student dashboard, so that results can be narrowed by lecturer name or date.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to build the GET /dashboard/student route and view, so that a student sees all consultations they have created or joined.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to persist the new consultation to MongoDB via the Consultation model, so that it is durably stored and retrievable.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to surface a user-friendly conflict error when a booking clashes, so that the student understands why their submission was rejected.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to enforce the max capacity limit when a student joins, so that the lecturer's capacity preference is never exceeded.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to display status badges (Open / Full / Cancelled) on each dashboard card, so that a student can see at a glance which sessions are joinable.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to validate the consultation datetime against the lecturer's availability window on submission, so that bookings outside available hours are rejected.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -382,6 +415,11 @@
       <color theme="0"/>
       <name val="Calibri (Body)"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="17">
     <fill>
@@ -412,11 +450,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA9DFBF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFAD7A0"/>
       </patternFill>
     </fill>
@@ -442,11 +475,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD5F5E3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFDEBD0"/>
       </patternFill>
     </fill>
@@ -467,6 +495,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="11">
     <border>
@@ -604,7 +644,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -614,7 +654,10 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -623,87 +666,95 @@
     <xf numFmtId="0" fontId="7" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF000000"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1001,132 +1052,132 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Y25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="15.6"/>
   <cols>
     <col min="1" max="1" width="12" style="1" customWidth="1"/>
     <col min="2" max="25" width="22" style="1" customWidth="1"/>
-    <col min="26" max="27" width="8.83203125" style="1" customWidth="1"/>
-    <col min="28" max="16384" width="8.83203125" style="1"/>
+    <col min="26" max="27" width="8.77734375" style="1" customWidth="1"/>
+    <col min="28" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+    <row r="1" spans="1:25" ht="28.05" customHeight="1">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
-      <c r="L1" s="21"/>
-      <c r="M1" s="21"/>
-      <c r="N1" s="21"/>
-      <c r="O1" s="21"/>
-      <c r="P1" s="21"/>
-      <c r="Q1" s="21"/>
-      <c r="R1" s="21"/>
-      <c r="S1" s="21"/>
-      <c r="T1" s="21"/>
-      <c r="U1" s="21"/>
-      <c r="V1" s="21"/>
-      <c r="W1" s="21"/>
-      <c r="X1" s="21"/>
-      <c r="Y1" s="21"/>
-    </row>
-    <row r="2" spans="1:25" s="11" customFormat="1" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="10"/>
-      <c r="B2" s="29" t="s">
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
+      <c r="O1" s="29"/>
+      <c r="P1" s="29"/>
+      <c r="Q1" s="29"/>
+      <c r="R1" s="29"/>
+      <c r="S1" s="29"/>
+      <c r="T1" s="29"/>
+      <c r="U1" s="29"/>
+      <c r="V1" s="29"/>
+      <c r="W1" s="29"/>
+      <c r="X1" s="29"/>
+      <c r="Y1" s="29"/>
+    </row>
+    <row r="2" spans="1:25" s="10" customFormat="1" ht="31.95" customHeight="1">
+      <c r="A2" s="9"/>
+      <c r="B2" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="23"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="22" t="s">
+      <c r="C2" s="20"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="24"/>
-      <c r="G2" s="12" t="s">
+      <c r="F2" s="25"/>
+      <c r="G2" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="22" t="s">
+      <c r="H2" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="23"/>
-      <c r="J2" s="23"/>
-      <c r="K2" s="23"/>
-      <c r="L2" s="24"/>
-      <c r="M2" s="22" t="s">
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="20"/>
+      <c r="L2" s="25"/>
+      <c r="M2" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="N2" s="23"/>
-      <c r="O2" s="23"/>
-      <c r="P2" s="24"/>
-      <c r="Q2" s="22" t="s">
+      <c r="N2" s="20"/>
+      <c r="O2" s="20"/>
+      <c r="P2" s="25"/>
+      <c r="Q2" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="R2" s="24"/>
-      <c r="S2" s="22" t="s">
+      <c r="R2" s="25"/>
+      <c r="S2" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="T2" s="24"/>
-      <c r="U2" s="30" t="s">
+      <c r="T2" s="25"/>
+      <c r="U2" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="V2" s="31"/>
-      <c r="W2" s="31"/>
-      <c r="X2" s="31"/>
-      <c r="Y2" s="31"/>
-    </row>
-    <row r="3" spans="1:25" s="18" customFormat="1" ht="230" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="19" t="s">
+      <c r="V2" s="33"/>
+      <c r="W2" s="33"/>
+      <c r="X2" s="33"/>
+      <c r="Y2" s="33"/>
+    </row>
+    <row r="3" spans="1:25" s="17" customFormat="1" ht="229.95" customHeight="1">
+      <c r="A3" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="23"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="22" t="s">
+      <c r="C3" s="20"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="24"/>
-      <c r="G3" s="12" t="s">
+      <c r="F3" s="25"/>
+      <c r="G3" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="22" t="s">
+      <c r="H3" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="I3" s="23"/>
-      <c r="J3" s="23"/>
-      <c r="K3" s="23"/>
-      <c r="L3" s="24"/>
-      <c r="M3" s="22" t="s">
+      <c r="I3" s="20"/>
+      <c r="J3" s="20"/>
+      <c r="K3" s="20"/>
+      <c r="L3" s="25"/>
+      <c r="M3" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="N3" s="23"/>
-      <c r="O3" s="23"/>
-      <c r="P3" s="24"/>
-      <c r="Q3" s="22" t="s">
+      <c r="N3" s="20"/>
+      <c r="O3" s="20"/>
+      <c r="P3" s="25"/>
+      <c r="Q3" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="R3" s="24"/>
-      <c r="S3" s="22" t="s">
+      <c r="R3" s="25"/>
+      <c r="S3" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="T3" s="24"/>
-      <c r="U3" s="33" t="s">
+      <c r="T3" s="25"/>
+      <c r="U3" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="V3" s="23"/>
-      <c r="W3" s="23"/>
-      <c r="X3" s="23"/>
-      <c r="Y3" s="23"/>
-    </row>
-    <row r="4" spans="1:25" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V3" s="20"/>
+      <c r="W3" s="20"/>
+      <c r="X3" s="20"/>
+      <c r="Y3" s="20"/>
+    </row>
+    <row r="4" spans="1:25" ht="36" customHeight="1">
       <c r="A4" s="2"/>
       <c r="B4" s="3" t="s">
         <v>17</v>
@@ -1201,7 +1252,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:25" ht="136" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:25" ht="136.05000000000001" customHeight="1">
       <c r="A5" s="4" t="s">
         <v>41</v>
       </c>
@@ -1278,39 +1329,39 @@
         <v>65</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="28" t="s">
+    <row r="6" spans="1:25" ht="16.05" customHeight="1">
+      <c r="A6" s="30" t="s">
         <v>66</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="B6" s="34" t="s">
         <v>67</v>
       </c>
-      <c r="C6" s="23"/>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="23"/>
-      <c r="G6" s="23"/>
-      <c r="H6" s="23"/>
-      <c r="I6" s="23"/>
-      <c r="J6" s="23"/>
-      <c r="K6" s="23"/>
-      <c r="L6" s="23"/>
-      <c r="M6" s="23"/>
-      <c r="N6" s="23"/>
-      <c r="O6" s="23"/>
-      <c r="P6" s="23"/>
-      <c r="Q6" s="23"/>
-      <c r="R6" s="23"/>
-      <c r="S6" s="23"/>
-      <c r="T6" s="23"/>
-      <c r="U6" s="23"/>
-      <c r="V6" s="23"/>
-      <c r="W6" s="23"/>
-      <c r="X6" s="23"/>
-      <c r="Y6" s="23"/>
-    </row>
-    <row r="7" spans="1:25" ht="123" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="26"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="20"/>
+      <c r="H6" s="20"/>
+      <c r="I6" s="20"/>
+      <c r="J6" s="20"/>
+      <c r="K6" s="20"/>
+      <c r="L6" s="20"/>
+      <c r="M6" s="20"/>
+      <c r="N6" s="20"/>
+      <c r="O6" s="20"/>
+      <c r="P6" s="20"/>
+      <c r="Q6" s="20"/>
+      <c r="R6" s="20"/>
+      <c r="S6" s="20"/>
+      <c r="T6" s="20"/>
+      <c r="U6" s="20"/>
+      <c r="V6" s="20"/>
+      <c r="W6" s="20"/>
+      <c r="X6" s="20"/>
+      <c r="Y6" s="20"/>
+    </row>
+    <row r="7" spans="1:25" ht="123" customHeight="1">
+      <c r="A7" s="22"/>
       <c r="B7" s="6" t="s">
         <v>68</v>
       </c>
@@ -1335,7 +1386,7 @@
       <c r="K7" s="6"/>
       <c r="L7" s="6"/>
       <c r="M7" s="6"/>
-      <c r="N7" s="13"/>
+      <c r="N7" s="12"/>
       <c r="O7" s="6"/>
       <c r="P7" s="6"/>
       <c r="Q7" s="6"/>
@@ -1345,11 +1396,11 @@
       <c r="U7" s="6"/>
       <c r="V7" s="6"/>
       <c r="W7" s="6"/>
-      <c r="X7" s="15"/>
-      <c r="Y7" s="15"/>
-    </row>
-    <row r="8" spans="1:25" ht="125" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="26"/>
+      <c r="X7" s="14"/>
+      <c r="Y7" s="14"/>
+    </row>
+    <row r="8" spans="1:25" ht="124.95" customHeight="1">
+      <c r="A8" s="22"/>
       <c r="B8" s="6" t="s">
         <v>86</v>
       </c>
@@ -1374,7 +1425,7 @@
       <c r="K8" s="6"/>
       <c r="L8" s="6"/>
       <c r="M8" s="6"/>
-      <c r="N8" s="14"/>
+      <c r="N8" s="13"/>
       <c r="O8" s="6"/>
       <c r="P8" s="6"/>
       <c r="Q8" s="6"/>
@@ -1384,11 +1435,11 @@
       <c r="U8" s="6"/>
       <c r="V8" s="6"/>
       <c r="W8" s="6"/>
-      <c r="X8" s="17"/>
-      <c r="Y8" s="16"/>
-    </row>
-    <row r="9" spans="1:25" ht="120" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="26"/>
+      <c r="X8" s="16"/>
+      <c r="Y8" s="15"/>
+    </row>
+    <row r="9" spans="1:25" ht="120" customHeight="1">
+      <c r="A9" s="22"/>
       <c r="B9" s="6" t="s">
         <v>79</v>
       </c>
@@ -1422,8 +1473,8 @@
       <c r="X9" s="6"/>
       <c r="Y9" s="6"/>
     </row>
-    <row r="10" spans="1:25" ht="78" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="27"/>
+    <row r="10" spans="1:25" ht="78" customHeight="1">
+      <c r="A10" s="23"/>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
       <c r="D10" s="6"/>
@@ -1449,433 +1500,447 @@
       <c r="X10" s="6"/>
       <c r="Y10" s="6"/>
     </row>
-    <row r="11" spans="1:25" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="25" t="s">
+    <row r="11" spans="1:25" ht="16.05" customHeight="1">
+      <c r="A11" s="38" t="s">
         <v>66</v>
       </c>
-      <c r="B11" s="36" t="s">
+      <c r="B11" s="41" t="s">
         <v>83</v>
       </c>
-      <c r="C11" s="23"/>
-      <c r="D11" s="23"/>
-      <c r="E11" s="23"/>
-      <c r="F11" s="23"/>
-      <c r="G11" s="23"/>
-      <c r="H11" s="23"/>
-      <c r="I11" s="23"/>
-      <c r="J11" s="23"/>
-      <c r="K11" s="23"/>
-      <c r="L11" s="23"/>
-      <c r="M11" s="23"/>
-      <c r="N11" s="23"/>
-      <c r="O11" s="23"/>
-      <c r="P11" s="23"/>
-      <c r="Q11" s="23"/>
-      <c r="R11" s="23"/>
-      <c r="S11" s="23"/>
-      <c r="T11" s="23"/>
-      <c r="U11" s="23"/>
-      <c r="V11" s="23"/>
-      <c r="W11" s="23"/>
-      <c r="X11" s="23"/>
-      <c r="Y11" s="23"/>
-    </row>
-    <row r="12" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="26"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
-      <c r="I12" s="7"/>
-      <c r="J12" s="7"/>
-      <c r="K12" s="7"/>
-      <c r="L12" s="7"/>
-      <c r="M12" s="7"/>
-      <c r="N12" s="7"/>
-      <c r="O12" s="7"/>
-      <c r="P12" s="7"/>
-      <c r="Q12" s="7"/>
-      <c r="R12" s="7"/>
-      <c r="S12" s="7"/>
-      <c r="T12" s="7"/>
-      <c r="U12" s="7"/>
-      <c r="V12" s="7"/>
-      <c r="W12" s="7"/>
-      <c r="X12" s="7"/>
-      <c r="Y12" s="7"/>
-    </row>
-    <row r="13" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="26"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
-      <c r="I13" s="7"/>
-      <c r="J13" s="7"/>
-      <c r="K13" s="7"/>
-      <c r="L13" s="7"/>
-      <c r="M13" s="7"/>
-      <c r="N13" s="7"/>
-      <c r="O13" s="7"/>
-      <c r="P13" s="7"/>
-      <c r="Q13" s="7"/>
-      <c r="R13" s="7"/>
-      <c r="S13" s="7"/>
-      <c r="T13" s="7"/>
-      <c r="U13" s="7"/>
-      <c r="V13" s="7"/>
-      <c r="W13" s="7"/>
-      <c r="X13" s="7"/>
-      <c r="Y13" s="7"/>
-    </row>
-    <row r="14" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="26"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
-      <c r="I14" s="7"/>
-      <c r="J14" s="7"/>
-      <c r="K14" s="7"/>
-      <c r="L14" s="7"/>
-      <c r="M14" s="7"/>
-      <c r="N14" s="7"/>
-      <c r="O14" s="7"/>
-      <c r="P14" s="7"/>
-      <c r="Q14" s="7"/>
-      <c r="R14" s="7"/>
-      <c r="S14" s="7"/>
-      <c r="T14" s="7"/>
-      <c r="U14" s="7"/>
-      <c r="V14" s="7"/>
-      <c r="W14" s="7"/>
-      <c r="X14" s="7"/>
-      <c r="Y14" s="7"/>
-    </row>
-    <row r="15" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="27"/>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
-      <c r="H15" s="7"/>
-      <c r="I15" s="7"/>
-      <c r="J15" s="7"/>
-      <c r="K15" s="7"/>
-      <c r="L15" s="7"/>
-      <c r="M15" s="7"/>
-      <c r="N15" s="7"/>
-      <c r="O15" s="7"/>
-      <c r="P15" s="7"/>
-      <c r="Q15" s="7"/>
-      <c r="R15" s="7"/>
-      <c r="S15" s="7"/>
-      <c r="T15" s="7"/>
-      <c r="U15" s="7"/>
-      <c r="V15" s="7"/>
-      <c r="W15" s="7"/>
-      <c r="X15" s="7"/>
-      <c r="Y15" s="7"/>
-    </row>
-    <row r="16" spans="1:25" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="38" t="s">
+      <c r="C11" s="42"/>
+      <c r="D11" s="42"/>
+      <c r="E11" s="42"/>
+      <c r="F11" s="42"/>
+      <c r="G11" s="42"/>
+      <c r="H11" s="42"/>
+      <c r="I11" s="42"/>
+      <c r="J11" s="42"/>
+      <c r="K11" s="42"/>
+      <c r="L11" s="42"/>
+      <c r="M11" s="42"/>
+      <c r="N11" s="42"/>
+      <c r="O11" s="42"/>
+      <c r="P11" s="42"/>
+      <c r="Q11" s="42"/>
+      <c r="R11" s="42"/>
+      <c r="S11" s="42"/>
+      <c r="T11" s="42"/>
+      <c r="U11" s="42"/>
+      <c r="V11" s="42"/>
+      <c r="W11" s="42"/>
+      <c r="X11" s="42"/>
+      <c r="Y11" s="42"/>
+    </row>
+    <row r="12" spans="1:25" ht="43.95" customHeight="1">
+      <c r="A12" s="39"/>
+      <c r="B12" s="36"/>
+      <c r="C12" s="36"/>
+      <c r="D12" s="36"/>
+      <c r="E12" s="36"/>
+      <c r="F12" s="36"/>
+      <c r="G12" s="36"/>
+      <c r="H12" s="37" t="s">
+        <v>88</v>
+      </c>
+      <c r="I12" s="37" t="s">
+        <v>89</v>
+      </c>
+      <c r="J12" s="37" t="s">
+        <v>90</v>
+      </c>
+      <c r="K12" s="37" t="s">
+        <v>91</v>
+      </c>
+      <c r="L12" s="37" t="s">
+        <v>92</v>
+      </c>
+      <c r="M12" s="37" t="s">
+        <v>93</v>
+      </c>
+      <c r="N12" s="36"/>
+      <c r="O12" s="36"/>
+      <c r="P12" s="36"/>
+      <c r="Q12" s="36"/>
+      <c r="R12" s="36"/>
+      <c r="S12" s="36"/>
+      <c r="T12" s="36"/>
+      <c r="U12" s="36"/>
+      <c r="V12" s="36"/>
+      <c r="W12" s="36"/>
+      <c r="X12" s="36"/>
+      <c r="Y12" s="36"/>
+    </row>
+    <row r="13" spans="1:25" ht="43.95" customHeight="1">
+      <c r="A13" s="39"/>
+      <c r="B13" s="36"/>
+      <c r="C13" s="36"/>
+      <c r="D13" s="36"/>
+      <c r="E13" s="36"/>
+      <c r="F13" s="36"/>
+      <c r="G13" s="36"/>
+      <c r="H13" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="I13" s="37" t="s">
+        <v>95</v>
+      </c>
+      <c r="J13" s="37" t="s">
+        <v>96</v>
+      </c>
+      <c r="K13" s="36"/>
+      <c r="L13" s="36"/>
+      <c r="M13" s="37" t="s">
+        <v>97</v>
+      </c>
+      <c r="N13" s="36"/>
+      <c r="O13" s="36"/>
+      <c r="P13" s="36"/>
+      <c r="Q13" s="36"/>
+      <c r="R13" s="36"/>
+      <c r="S13" s="36"/>
+      <c r="T13" s="36"/>
+      <c r="U13" s="36"/>
+      <c r="V13" s="36"/>
+      <c r="W13" s="36"/>
+      <c r="X13" s="36"/>
+      <c r="Y13" s="36"/>
+    </row>
+    <row r="14" spans="1:25" ht="43.95" customHeight="1">
+      <c r="A14" s="39"/>
+      <c r="B14" s="36"/>
+      <c r="C14" s="36"/>
+      <c r="D14" s="36"/>
+      <c r="E14" s="36"/>
+      <c r="F14" s="36"/>
+      <c r="G14" s="36"/>
+      <c r="H14" s="37" t="s">
+        <v>98</v>
+      </c>
+      <c r="I14" s="36"/>
+      <c r="J14" s="36"/>
+      <c r="K14" s="36"/>
+      <c r="L14" s="36"/>
+      <c r="M14" s="36"/>
+      <c r="N14" s="36"/>
+      <c r="O14" s="36"/>
+      <c r="P14" s="36"/>
+      <c r="Q14" s="36"/>
+      <c r="R14" s="36"/>
+      <c r="S14" s="36"/>
+      <c r="T14" s="36"/>
+      <c r="U14" s="36"/>
+      <c r="V14" s="36"/>
+      <c r="W14" s="36"/>
+      <c r="X14" s="36"/>
+      <c r="Y14" s="36"/>
+    </row>
+    <row r="15" spans="1:25" ht="43.95" customHeight="1">
+      <c r="A15" s="40"/>
+      <c r="B15" s="36"/>
+      <c r="C15" s="36"/>
+      <c r="D15" s="36"/>
+      <c r="E15" s="36"/>
+      <c r="F15" s="36"/>
+      <c r="G15" s="36"/>
+      <c r="H15" s="36"/>
+      <c r="I15" s="36"/>
+      <c r="J15" s="36"/>
+      <c r="K15" s="36"/>
+      <c r="L15" s="36"/>
+      <c r="M15" s="36"/>
+      <c r="N15" s="36"/>
+      <c r="O15" s="36"/>
+      <c r="P15" s="36"/>
+      <c r="Q15" s="36"/>
+      <c r="R15" s="36"/>
+      <c r="S15" s="36"/>
+      <c r="T15" s="36"/>
+      <c r="U15" s="36"/>
+      <c r="V15" s="36"/>
+      <c r="W15" s="36"/>
+      <c r="X15" s="36"/>
+      <c r="Y15" s="36"/>
+    </row>
+    <row r="16" spans="1:25" ht="16.05" customHeight="1">
+      <c r="A16" s="27" t="s">
         <v>66</v>
       </c>
-      <c r="B16" s="37" t="s">
+      <c r="B16" s="26" t="s">
         <v>84</v>
       </c>
-      <c r="C16" s="23"/>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="23"/>
-      <c r="I16" s="23"/>
-      <c r="J16" s="23"/>
-      <c r="K16" s="23"/>
-      <c r="L16" s="23"/>
-      <c r="M16" s="23"/>
-      <c r="N16" s="23"/>
-      <c r="O16" s="23"/>
-      <c r="P16" s="23"/>
-      <c r="Q16" s="23"/>
-      <c r="R16" s="23"/>
-      <c r="S16" s="23"/>
-      <c r="T16" s="23"/>
-      <c r="U16" s="23"/>
-      <c r="V16" s="23"/>
-      <c r="W16" s="23"/>
-      <c r="X16" s="23"/>
-      <c r="Y16" s="23"/>
-    </row>
-    <row r="17" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="26"/>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="8"/>
-      <c r="I17" s="8"/>
-      <c r="J17" s="8"/>
-      <c r="K17" s="8"/>
-      <c r="L17" s="8"/>
-      <c r="M17" s="8"/>
-      <c r="N17" s="8"/>
-      <c r="O17" s="8"/>
-      <c r="P17" s="8"/>
-      <c r="Q17" s="8"/>
-      <c r="R17" s="8"/>
-      <c r="S17" s="8"/>
-      <c r="T17" s="8"/>
-      <c r="U17" s="8"/>
-      <c r="V17" s="8"/>
-      <c r="W17" s="8"/>
-      <c r="X17" s="8"/>
-      <c r="Y17" s="8"/>
-    </row>
-    <row r="18" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="26"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
-      <c r="I18" s="8"/>
-      <c r="J18" s="8"/>
-      <c r="K18" s="8"/>
-      <c r="L18" s="8"/>
-      <c r="M18" s="8"/>
-      <c r="N18" s="8"/>
-      <c r="O18" s="8"/>
-      <c r="P18" s="8"/>
-      <c r="Q18" s="8"/>
-      <c r="R18" s="8"/>
-      <c r="S18" s="8"/>
-      <c r="T18" s="8"/>
-      <c r="U18" s="8"/>
-      <c r="V18" s="8"/>
-      <c r="W18" s="8"/>
-      <c r="X18" s="8"/>
-      <c r="Y18" s="8"/>
-    </row>
-    <row r="19" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="26"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
-      <c r="J19" s="8"/>
-      <c r="K19" s="8"/>
-      <c r="L19" s="8"/>
-      <c r="M19" s="8"/>
-      <c r="N19" s="8"/>
-      <c r="O19" s="8"/>
-      <c r="P19" s="8"/>
-      <c r="Q19" s="8"/>
-      <c r="R19" s="8"/>
-      <c r="S19" s="8"/>
-      <c r="T19" s="8"/>
-      <c r="U19" s="8"/>
-      <c r="V19" s="8"/>
-      <c r="W19" s="8"/>
-      <c r="X19" s="8"/>
-      <c r="Y19" s="8"/>
-    </row>
-    <row r="20" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="27"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="8"/>
-      <c r="K20" s="8"/>
-      <c r="L20" s="8"/>
-      <c r="M20" s="8"/>
-      <c r="N20" s="8"/>
-      <c r="O20" s="8"/>
-      <c r="P20" s="8"/>
-      <c r="Q20" s="8"/>
-      <c r="R20" s="8"/>
-      <c r="S20" s="8"/>
-      <c r="T20" s="8"/>
-      <c r="U20" s="8"/>
-      <c r="V20" s="8"/>
-      <c r="W20" s="8"/>
-      <c r="X20" s="8"/>
-      <c r="Y20" s="8"/>
-    </row>
-    <row r="21" spans="1:25" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="35" t="s">
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="20"/>
+      <c r="I16" s="20"/>
+      <c r="J16" s="20"/>
+      <c r="K16" s="20"/>
+      <c r="L16" s="20"/>
+      <c r="M16" s="20"/>
+      <c r="N16" s="20"/>
+      <c r="O16" s="20"/>
+      <c r="P16" s="20"/>
+      <c r="Q16" s="20"/>
+      <c r="R16" s="20"/>
+      <c r="S16" s="20"/>
+      <c r="T16" s="20"/>
+      <c r="U16" s="20"/>
+      <c r="V16" s="20"/>
+      <c r="W16" s="20"/>
+      <c r="X16" s="20"/>
+      <c r="Y16" s="20"/>
+    </row>
+    <row r="17" spans="1:25" ht="43.95" customHeight="1">
+      <c r="A17" s="22"/>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="7"/>
+      <c r="J17" s="7"/>
+      <c r="K17" s="7"/>
+      <c r="L17" s="7"/>
+      <c r="M17" s="7"/>
+      <c r="N17" s="7"/>
+      <c r="O17" s="7"/>
+      <c r="P17" s="7"/>
+      <c r="Q17" s="7"/>
+      <c r="R17" s="7"/>
+      <c r="S17" s="7"/>
+      <c r="T17" s="7"/>
+      <c r="U17" s="7"/>
+      <c r="V17" s="7"/>
+      <c r="W17" s="7"/>
+      <c r="X17" s="7"/>
+      <c r="Y17" s="7"/>
+    </row>
+    <row r="18" spans="1:25" ht="43.95" customHeight="1">
+      <c r="A18" s="22"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="7"/>
+      <c r="I18" s="7"/>
+      <c r="J18" s="7"/>
+      <c r="K18" s="7"/>
+      <c r="L18" s="7"/>
+      <c r="M18" s="7"/>
+      <c r="N18" s="7"/>
+      <c r="O18" s="7"/>
+      <c r="P18" s="7"/>
+      <c r="Q18" s="7"/>
+      <c r="R18" s="7"/>
+      <c r="S18" s="7"/>
+      <c r="T18" s="7"/>
+      <c r="U18" s="7"/>
+      <c r="V18" s="7"/>
+      <c r="W18" s="7"/>
+      <c r="X18" s="7"/>
+      <c r="Y18" s="7"/>
+    </row>
+    <row r="19" spans="1:25" ht="43.95" customHeight="1">
+      <c r="A19" s="22"/>
+      <c r="B19" s="7"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="7"/>
+      <c r="J19" s="7"/>
+      <c r="K19" s="7"/>
+      <c r="L19" s="7"/>
+      <c r="M19" s="7"/>
+      <c r="N19" s="7"/>
+      <c r="O19" s="7"/>
+      <c r="P19" s="7"/>
+      <c r="Q19" s="7"/>
+      <c r="R19" s="7"/>
+      <c r="S19" s="7"/>
+      <c r="T19" s="7"/>
+      <c r="U19" s="7"/>
+      <c r="V19" s="7"/>
+      <c r="W19" s="7"/>
+      <c r="X19" s="7"/>
+      <c r="Y19" s="7"/>
+    </row>
+    <row r="20" spans="1:25" ht="43.95" customHeight="1">
+      <c r="A20" s="23"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="7"/>
+      <c r="H20" s="7"/>
+      <c r="I20" s="7"/>
+      <c r="J20" s="7"/>
+      <c r="K20" s="7"/>
+      <c r="L20" s="7"/>
+      <c r="M20" s="7"/>
+      <c r="N20" s="7"/>
+      <c r="O20" s="7"/>
+      <c r="P20" s="7"/>
+      <c r="Q20" s="7"/>
+      <c r="R20" s="7"/>
+      <c r="S20" s="7"/>
+      <c r="T20" s="7"/>
+      <c r="U20" s="7"/>
+      <c r="V20" s="7"/>
+      <c r="W20" s="7"/>
+      <c r="X20" s="7"/>
+      <c r="Y20" s="7"/>
+    </row>
+    <row r="21" spans="1:25" ht="16.05" customHeight="1">
+      <c r="A21" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="B21" s="34" t="s">
+      <c r="B21" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="C21" s="23"/>
-      <c r="D21" s="23"/>
-      <c r="E21" s="23"/>
-      <c r="F21" s="23"/>
-      <c r="G21" s="23"/>
-      <c r="H21" s="23"/>
-      <c r="I21" s="23"/>
-      <c r="J21" s="23"/>
-      <c r="K21" s="23"/>
-      <c r="L21" s="23"/>
-      <c r="M21" s="23"/>
-      <c r="N21" s="23"/>
-      <c r="O21" s="23"/>
-      <c r="P21" s="23"/>
-      <c r="Q21" s="23"/>
-      <c r="R21" s="23"/>
-      <c r="S21" s="23"/>
-      <c r="T21" s="23"/>
-      <c r="U21" s="23"/>
-      <c r="V21" s="23"/>
-      <c r="W21" s="23"/>
-      <c r="X21" s="23"/>
-      <c r="Y21" s="23"/>
-    </row>
-    <row r="22" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="26"/>
-      <c r="B22" s="9"/>
-      <c r="C22" s="9"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
-      <c r="G22" s="9"/>
-      <c r="H22" s="9"/>
-      <c r="I22" s="9"/>
-      <c r="J22" s="9"/>
-      <c r="K22" s="9"/>
-      <c r="L22" s="9"/>
-      <c r="M22" s="9"/>
-      <c r="N22" s="9"/>
-      <c r="O22" s="9"/>
-      <c r="P22" s="9"/>
-      <c r="Q22" s="9"/>
-      <c r="R22" s="9"/>
-      <c r="S22" s="9"/>
-      <c r="T22" s="9"/>
-      <c r="U22" s="9"/>
-      <c r="V22" s="9"/>
-      <c r="W22" s="9"/>
-      <c r="X22" s="9"/>
-      <c r="Y22" s="9"/>
-    </row>
-    <row r="23" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="26"/>
-      <c r="B23" s="9"/>
-      <c r="C23" s="9"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
-      <c r="G23" s="9"/>
-      <c r="H23" s="9"/>
-      <c r="I23" s="9"/>
-      <c r="J23" s="9"/>
-      <c r="K23" s="9"/>
-      <c r="L23" s="9"/>
-      <c r="M23" s="9"/>
-      <c r="N23" s="9"/>
-      <c r="O23" s="9"/>
-      <c r="P23" s="9"/>
-      <c r="Q23" s="9"/>
-      <c r="R23" s="9"/>
-      <c r="S23" s="9"/>
-      <c r="T23" s="9"/>
-      <c r="U23" s="9"/>
-      <c r="V23" s="9"/>
-      <c r="W23" s="9"/>
-      <c r="X23" s="9"/>
-      <c r="Y23" s="9"/>
-    </row>
-    <row r="24" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="26"/>
-      <c r="B24" s="9"/>
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="9"/>
-      <c r="H24" s="9"/>
-      <c r="I24" s="9"/>
-      <c r="J24" s="9"/>
-      <c r="K24" s="9"/>
-      <c r="L24" s="9"/>
-      <c r="M24" s="9"/>
-      <c r="N24" s="9"/>
-      <c r="O24" s="9"/>
-      <c r="P24" s="9"/>
-      <c r="Q24" s="9"/>
-      <c r="R24" s="9"/>
-      <c r="S24" s="9"/>
-      <c r="T24" s="9"/>
-      <c r="U24" s="9"/>
-      <c r="V24" s="9"/>
-      <c r="W24" s="9"/>
-      <c r="X24" s="9"/>
-      <c r="Y24" s="9"/>
-    </row>
-    <row r="25" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="27"/>
-      <c r="B25" s="9"/>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="9"/>
-      <c r="H25" s="9"/>
-      <c r="I25" s="9"/>
-      <c r="J25" s="9"/>
-      <c r="K25" s="9"/>
-      <c r="L25" s="9"/>
-      <c r="M25" s="9"/>
-      <c r="N25" s="9"/>
-      <c r="O25" s="9"/>
-      <c r="P25" s="9"/>
-      <c r="Q25" s="9"/>
-      <c r="R25" s="9"/>
-      <c r="S25" s="9"/>
-      <c r="T25" s="9"/>
-      <c r="U25" s="9"/>
-      <c r="V25" s="9"/>
-      <c r="W25" s="9"/>
-      <c r="X25" s="9"/>
-      <c r="Y25" s="9"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="20"/>
+      <c r="H21" s="20"/>
+      <c r="I21" s="20"/>
+      <c r="J21" s="20"/>
+      <c r="K21" s="20"/>
+      <c r="L21" s="20"/>
+      <c r="M21" s="20"/>
+      <c r="N21" s="20"/>
+      <c r="O21" s="20"/>
+      <c r="P21" s="20"/>
+      <c r="Q21" s="20"/>
+      <c r="R21" s="20"/>
+      <c r="S21" s="20"/>
+      <c r="T21" s="20"/>
+      <c r="U21" s="20"/>
+      <c r="V21" s="20"/>
+      <c r="W21" s="20"/>
+      <c r="X21" s="20"/>
+      <c r="Y21" s="20"/>
+    </row>
+    <row r="22" spans="1:25" ht="43.95" customHeight="1">
+      <c r="A22" s="22"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="8"/>
+      <c r="I22" s="8"/>
+      <c r="J22" s="8"/>
+      <c r="K22" s="8"/>
+      <c r="L22" s="8"/>
+      <c r="M22" s="8"/>
+      <c r="N22" s="8"/>
+      <c r="O22" s="8"/>
+      <c r="P22" s="8"/>
+      <c r="Q22" s="8"/>
+      <c r="R22" s="8"/>
+      <c r="S22" s="8"/>
+      <c r="T22" s="8"/>
+      <c r="U22" s="8"/>
+      <c r="V22" s="8"/>
+      <c r="W22" s="8"/>
+      <c r="X22" s="8"/>
+      <c r="Y22" s="8"/>
+    </row>
+    <row r="23" spans="1:25" ht="43.95" customHeight="1">
+      <c r="A23" s="22"/>
+      <c r="B23" s="8"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="8"/>
+      <c r="J23" s="8"/>
+      <c r="K23" s="8"/>
+      <c r="L23" s="8"/>
+      <c r="M23" s="8"/>
+      <c r="N23" s="8"/>
+      <c r="O23" s="8"/>
+      <c r="P23" s="8"/>
+      <c r="Q23" s="8"/>
+      <c r="R23" s="8"/>
+      <c r="S23" s="8"/>
+      <c r="T23" s="8"/>
+      <c r="U23" s="8"/>
+      <c r="V23" s="8"/>
+      <c r="W23" s="8"/>
+      <c r="X23" s="8"/>
+      <c r="Y23" s="8"/>
+    </row>
+    <row r="24" spans="1:25" ht="43.95" customHeight="1">
+      <c r="A24" s="22"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
+      <c r="G24" s="8"/>
+      <c r="H24" s="8"/>
+      <c r="I24" s="8"/>
+      <c r="J24" s="8"/>
+      <c r="K24" s="8"/>
+      <c r="L24" s="8"/>
+      <c r="M24" s="8"/>
+      <c r="N24" s="8"/>
+      <c r="O24" s="8"/>
+      <c r="P24" s="8"/>
+      <c r="Q24" s="8"/>
+      <c r="R24" s="8"/>
+      <c r="S24" s="8"/>
+      <c r="T24" s="8"/>
+      <c r="U24" s="8"/>
+      <c r="V24" s="8"/>
+      <c r="W24" s="8"/>
+      <c r="X24" s="8"/>
+      <c r="Y24" s="8"/>
+    </row>
+    <row r="25" spans="1:25" ht="43.95" customHeight="1">
+      <c r="A25" s="23"/>
+      <c r="B25" s="8"/>
+      <c r="C25" s="8"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="8"/>
+      <c r="I25" s="8"/>
+      <c r="J25" s="8"/>
+      <c r="K25" s="8"/>
+      <c r="L25" s="8"/>
+      <c r="M25" s="8"/>
+      <c r="N25" s="8"/>
+      <c r="O25" s="8"/>
+      <c r="P25" s="8"/>
+      <c r="Q25" s="8"/>
+      <c r="R25" s="8"/>
+      <c r="S25" s="8"/>
+      <c r="T25" s="8"/>
+      <c r="U25" s="8"/>
+      <c r="V25" s="8"/>
+      <c r="W25" s="8"/>
+      <c r="X25" s="8"/>
+      <c r="Y25" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="23">
-    <mergeCell ref="B21:Y21"/>
-    <mergeCell ref="A21:A25"/>
-    <mergeCell ref="Q3:R3"/>
-    <mergeCell ref="M3:P3"/>
-    <mergeCell ref="B11:Y11"/>
-    <mergeCell ref="S3:T3"/>
-    <mergeCell ref="B16:Y16"/>
-    <mergeCell ref="A16:A20"/>
     <mergeCell ref="A1:Y1"/>
     <mergeCell ref="M2:P2"/>
     <mergeCell ref="A11:A15"/>
@@ -1891,6 +1956,14 @@
     <mergeCell ref="B6:Y6"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="U3:Y3"/>
+    <mergeCell ref="B21:Y21"/>
+    <mergeCell ref="A21:A25"/>
+    <mergeCell ref="Q3:R3"/>
+    <mergeCell ref="M3:P3"/>
+    <mergeCell ref="B11:Y11"/>
+    <mergeCell ref="S3:T3"/>
+    <mergeCell ref="B16:Y16"/>
+    <mergeCell ref="A16:A20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(documentation): add sprint 2 retrospective and sprint 3 scrum board and update user story map
</commit_message>
<xml_diff>
--- a/documentation/user_story_mapping/user_story_map.xlsx
+++ b/documentation/user_story_mapping/user_story_map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\khela\ELEN4010 Group Lab\2026-group-lab-001\documentation\user_story_mapping\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E24A244B-9F51-4F49-8C37-61DA4A67C6E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D98BB366-5AF1-4B52-BEB2-DB536A596CE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Story Map" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="112">
   <si>
     <t>Consultation Scheduler — User Story Map</t>
   </si>
@@ -319,6 +319,45 @@
   </si>
   <si>
     <t>As a developer, I want to validate the consultation datetime against the lecturer's availability window on submission, so that bookings outside available hours are rejected.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to build the GET /dashboard/lecturer route and view, so that a lecturer sees all upcoming consultations they are hosting.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to display attendee count and remaining capacity on each lecturer dashboard card, so that the lecturer can see at a glance how full each session is.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to surface a 'No upcoming sessions' empty state on the lecturer dashboard when no consultations are scheduled, so that the view is informative rather than blank.</t>
+  </si>
+  <si>
+    <t>Completed in Sprint 2.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to build a GET /consultations/:id/attendees endpoint, so that attendee data is available for rendering on the lecturer dashboard.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to render the attendee name list on each lecturer dashboard consultation card, so that the lecturer can identify who is attending each session.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to build a DELETE /consultations/:id route restricted to the organising student, so that they can cancel a consultation they created.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to build a DELETE /consultations/:id/cancel route for lecturers, so that they can cancel any consultation on their schedule.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to update the consultation status to Cancelled and persist the change to MongoDB, so that all views reflect the cancellation immediately.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to build an activity logging middleware, so that every mutating request is captured with the user, action type, and timestamp.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to persist each log entry as a document in a dedicated ActivityLog MongoDB collection, so that audit records are durable and queryable.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to build a GET /admin/logs route and paginated view, so that an administrator can browse the full activity log.</t>
+  </si>
+  <si>
+    <t>As a developer, I want to add user and date filters to the activity log query, so that the admin can narrow the audit trail by actor or time range.</t>
   </si>
 </sst>
 </file>
@@ -690,32 +729,31 @@
     <xf numFmtId="0" fontId="11" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -729,21 +767,22 @@
     <xf numFmtId="0" fontId="9" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1061,121 +1100,121 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="28.05" customHeight="1">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-      <c r="L1" s="29"/>
-      <c r="M1" s="29"/>
-      <c r="N1" s="29"/>
-      <c r="O1" s="29"/>
-      <c r="P1" s="29"/>
-      <c r="Q1" s="29"/>
-      <c r="R1" s="29"/>
-      <c r="S1" s="29"/>
-      <c r="T1" s="29"/>
-      <c r="U1" s="29"/>
-      <c r="V1" s="29"/>
-      <c r="W1" s="29"/>
-      <c r="X1" s="29"/>
-      <c r="Y1" s="29"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
+      <c r="M1" s="22"/>
+      <c r="N1" s="22"/>
+      <c r="O1" s="22"/>
+      <c r="P1" s="22"/>
+      <c r="Q1" s="22"/>
+      <c r="R1" s="22"/>
+      <c r="S1" s="22"/>
+      <c r="T1" s="22"/>
+      <c r="U1" s="22"/>
+      <c r="V1" s="22"/>
+      <c r="W1" s="22"/>
+      <c r="X1" s="22"/>
+      <c r="Y1" s="22"/>
     </row>
     <row r="2" spans="1:25" s="10" customFormat="1" ht="31.95" customHeight="1">
       <c r="A2" s="9"/>
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="20"/>
+      <c r="C2" s="24"/>
       <c r="D2" s="25"/>
-      <c r="E2" s="24" t="s">
+      <c r="E2" s="23" t="s">
         <v>2</v>
       </c>
       <c r="F2" s="25"/>
       <c r="G2" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="24" t="s">
+      <c r="H2" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="20"/>
-      <c r="J2" s="20"/>
-      <c r="K2" s="20"/>
+      <c r="I2" s="24"/>
+      <c r="J2" s="24"/>
+      <c r="K2" s="24"/>
       <c r="L2" s="25"/>
-      <c r="M2" s="24" t="s">
+      <c r="M2" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="N2" s="20"/>
-      <c r="O2" s="20"/>
+      <c r="N2" s="24"/>
+      <c r="O2" s="24"/>
       <c r="P2" s="25"/>
-      <c r="Q2" s="24" t="s">
+      <c r="Q2" s="23" t="s">
         <v>6</v>
       </c>
       <c r="R2" s="25"/>
-      <c r="S2" s="24" t="s">
+      <c r="S2" s="23" t="s">
         <v>7</v>
       </c>
       <c r="T2" s="25"/>
-      <c r="U2" s="32" t="s">
+      <c r="U2" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="V2" s="33"/>
-      <c r="W2" s="33"/>
-      <c r="X2" s="33"/>
-      <c r="Y2" s="33"/>
+      <c r="V2" s="34"/>
+      <c r="W2" s="34"/>
+      <c r="X2" s="34"/>
+      <c r="Y2" s="34"/>
     </row>
     <row r="3" spans="1:25" s="17" customFormat="1" ht="229.95" customHeight="1">
       <c r="A3" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="B3" s="31" t="s">
+      <c r="B3" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="20"/>
+      <c r="C3" s="24"/>
       <c r="D3" s="25"/>
-      <c r="E3" s="24" t="s">
+      <c r="E3" s="23" t="s">
         <v>10</v>
       </c>
       <c r="F3" s="25"/>
       <c r="G3" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="24" t="s">
+      <c r="H3" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="I3" s="20"/>
-      <c r="J3" s="20"/>
-      <c r="K3" s="20"/>
+      <c r="I3" s="24"/>
+      <c r="J3" s="24"/>
+      <c r="K3" s="24"/>
       <c r="L3" s="25"/>
-      <c r="M3" s="24" t="s">
+      <c r="M3" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="N3" s="20"/>
-      <c r="O3" s="20"/>
+      <c r="N3" s="24"/>
+      <c r="O3" s="24"/>
       <c r="P3" s="25"/>
-      <c r="Q3" s="24" t="s">
+      <c r="Q3" s="23" t="s">
         <v>14</v>
       </c>
       <c r="R3" s="25"/>
-      <c r="S3" s="24" t="s">
+      <c r="S3" s="23" t="s">
         <v>15</v>
       </c>
       <c r="T3" s="25"/>
-      <c r="U3" s="35" t="s">
+      <c r="U3" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="V3" s="20"/>
-      <c r="W3" s="20"/>
-      <c r="X3" s="20"/>
-      <c r="Y3" s="20"/>
+      <c r="V3" s="24"/>
+      <c r="W3" s="24"/>
+      <c r="X3" s="24"/>
+      <c r="Y3" s="24"/>
     </row>
     <row r="4" spans="1:25" ht="36" customHeight="1">
       <c r="A4" s="2"/>
@@ -1330,38 +1369,38 @@
       </c>
     </row>
     <row r="6" spans="1:25" ht="16.05" customHeight="1">
-      <c r="A6" s="30" t="s">
+      <c r="A6" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="B6" s="34" t="s">
+      <c r="B6" s="35" t="s">
         <v>67</v>
       </c>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="20"/>
-      <c r="H6" s="20"/>
-      <c r="I6" s="20"/>
-      <c r="J6" s="20"/>
-      <c r="K6" s="20"/>
-      <c r="L6" s="20"/>
-      <c r="M6" s="20"/>
-      <c r="N6" s="20"/>
-      <c r="O6" s="20"/>
-      <c r="P6" s="20"/>
-      <c r="Q6" s="20"/>
-      <c r="R6" s="20"/>
-      <c r="S6" s="20"/>
-      <c r="T6" s="20"/>
-      <c r="U6" s="20"/>
-      <c r="V6" s="20"/>
-      <c r="W6" s="20"/>
-      <c r="X6" s="20"/>
-      <c r="Y6" s="20"/>
+      <c r="C6" s="24"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="24"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="24"/>
+      <c r="H6" s="24"/>
+      <c r="I6" s="24"/>
+      <c r="J6" s="24"/>
+      <c r="K6" s="24"/>
+      <c r="L6" s="24"/>
+      <c r="M6" s="24"/>
+      <c r="N6" s="24"/>
+      <c r="O6" s="24"/>
+      <c r="P6" s="24"/>
+      <c r="Q6" s="24"/>
+      <c r="R6" s="24"/>
+      <c r="S6" s="24"/>
+      <c r="T6" s="24"/>
+      <c r="U6" s="24"/>
+      <c r="V6" s="24"/>
+      <c r="W6" s="24"/>
+      <c r="X6" s="24"/>
+      <c r="Y6" s="24"/>
     </row>
     <row r="7" spans="1:25" ht="123" customHeight="1">
-      <c r="A7" s="22"/>
+      <c r="A7" s="30"/>
       <c r="B7" s="6" t="s">
         <v>68</v>
       </c>
@@ -1400,7 +1439,7 @@
       <c r="Y7" s="14"/>
     </row>
     <row r="8" spans="1:25" ht="124.95" customHeight="1">
-      <c r="A8" s="22"/>
+      <c r="A8" s="30"/>
       <c r="B8" s="6" t="s">
         <v>86</v>
       </c>
@@ -1439,7 +1478,7 @@
       <c r="Y8" s="15"/>
     </row>
     <row r="9" spans="1:25" ht="120" customHeight="1">
-      <c r="A9" s="22"/>
+      <c r="A9" s="30"/>
       <c r="B9" s="6" t="s">
         <v>79</v>
       </c>
@@ -1474,7 +1513,7 @@
       <c r="Y9" s="6"/>
     </row>
     <row r="10" spans="1:25" ht="78" customHeight="1">
-      <c r="A10" s="23"/>
+      <c r="A10" s="31"/>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
       <c r="D10" s="6"/>
@@ -1501,199 +1540,199 @@
       <c r="Y10" s="6"/>
     </row>
     <row r="11" spans="1:25" ht="16.05" customHeight="1">
-      <c r="A11" s="38" t="s">
+      <c r="A11" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="B11" s="41" t="s">
+      <c r="B11" s="39" t="s">
         <v>83</v>
       </c>
-      <c r="C11" s="42"/>
-      <c r="D11" s="42"/>
-      <c r="E11" s="42"/>
-      <c r="F11" s="42"/>
-      <c r="G11" s="42"/>
-      <c r="H11" s="42"/>
-      <c r="I11" s="42"/>
-      <c r="J11" s="42"/>
-      <c r="K11" s="42"/>
-      <c r="L11" s="42"/>
-      <c r="M11" s="42"/>
-      <c r="N11" s="42"/>
-      <c r="O11" s="42"/>
-      <c r="P11" s="42"/>
-      <c r="Q11" s="42"/>
-      <c r="R11" s="42"/>
-      <c r="S11" s="42"/>
-      <c r="T11" s="42"/>
-      <c r="U11" s="42"/>
-      <c r="V11" s="42"/>
-      <c r="W11" s="42"/>
-      <c r="X11" s="42"/>
-      <c r="Y11" s="42"/>
+      <c r="C11" s="40"/>
+      <c r="D11" s="40"/>
+      <c r="E11" s="40"/>
+      <c r="F11" s="40"/>
+      <c r="G11" s="40"/>
+      <c r="H11" s="40"/>
+      <c r="I11" s="40"/>
+      <c r="J11" s="40"/>
+      <c r="K11" s="40"/>
+      <c r="L11" s="40"/>
+      <c r="M11" s="40"/>
+      <c r="N11" s="40"/>
+      <c r="O11" s="40"/>
+      <c r="P11" s="40"/>
+      <c r="Q11" s="40"/>
+      <c r="R11" s="40"/>
+      <c r="S11" s="40"/>
+      <c r="T11" s="40"/>
+      <c r="U11" s="40"/>
+      <c r="V11" s="40"/>
+      <c r="W11" s="40"/>
+      <c r="X11" s="40"/>
+      <c r="Y11" s="40"/>
     </row>
     <row r="12" spans="1:25" ht="43.95" customHeight="1">
-      <c r="A12" s="39"/>
-      <c r="B12" s="36"/>
-      <c r="C12" s="36"/>
-      <c r="D12" s="36"/>
-      <c r="E12" s="36"/>
-      <c r="F12" s="36"/>
-      <c r="G12" s="36"/>
-      <c r="H12" s="37" t="s">
+      <c r="A12" s="27"/>
+      <c r="B12" s="19"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
+      <c r="G12" s="19"/>
+      <c r="H12" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="I12" s="37" t="s">
+      <c r="I12" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="J12" s="37" t="s">
+      <c r="J12" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="K12" s="37" t="s">
+      <c r="K12" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="L12" s="37" t="s">
+      <c r="L12" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="M12" s="37" t="s">
+      <c r="M12" s="20" t="s">
         <v>93</v>
       </c>
-      <c r="N12" s="36"/>
-      <c r="O12" s="36"/>
-      <c r="P12" s="36"/>
-      <c r="Q12" s="36"/>
-      <c r="R12" s="36"/>
-      <c r="S12" s="36"/>
-      <c r="T12" s="36"/>
-      <c r="U12" s="36"/>
-      <c r="V12" s="36"/>
-      <c r="W12" s="36"/>
-      <c r="X12" s="36"/>
-      <c r="Y12" s="36"/>
+      <c r="N12" s="19"/>
+      <c r="O12" s="19"/>
+      <c r="P12" s="19"/>
+      <c r="Q12" s="19"/>
+      <c r="R12" s="19"/>
+      <c r="S12" s="19"/>
+      <c r="T12" s="19"/>
+      <c r="U12" s="19"/>
+      <c r="V12" s="19"/>
+      <c r="W12" s="19"/>
+      <c r="X12" s="19"/>
+      <c r="Y12" s="19"/>
     </row>
     <row r="13" spans="1:25" ht="43.95" customHeight="1">
-      <c r="A13" s="39"/>
-      <c r="B13" s="36"/>
-      <c r="C13" s="36"/>
-      <c r="D13" s="36"/>
-      <c r="E13" s="36"/>
-      <c r="F13" s="36"/>
-      <c r="G13" s="36"/>
-      <c r="H13" s="37" t="s">
+      <c r="A13" s="27"/>
+      <c r="B13" s="19"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
+      <c r="G13" s="19"/>
+      <c r="H13" s="20" t="s">
         <v>94</v>
       </c>
-      <c r="I13" s="37" t="s">
+      <c r="I13" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="J13" s="37" t="s">
+      <c r="J13" s="20" t="s">
         <v>96</v>
       </c>
-      <c r="K13" s="36"/>
-      <c r="L13" s="36"/>
-      <c r="M13" s="37" t="s">
+      <c r="K13" s="19"/>
+      <c r="L13" s="19"/>
+      <c r="M13" s="20" t="s">
         <v>97</v>
       </c>
-      <c r="N13" s="36"/>
-      <c r="O13" s="36"/>
-      <c r="P13" s="36"/>
-      <c r="Q13" s="36"/>
-      <c r="R13" s="36"/>
-      <c r="S13" s="36"/>
-      <c r="T13" s="36"/>
-      <c r="U13" s="36"/>
-      <c r="V13" s="36"/>
-      <c r="W13" s="36"/>
-      <c r="X13" s="36"/>
-      <c r="Y13" s="36"/>
+      <c r="N13" s="19"/>
+      <c r="O13" s="19"/>
+      <c r="P13" s="19"/>
+      <c r="Q13" s="19"/>
+      <c r="R13" s="19"/>
+      <c r="S13" s="19"/>
+      <c r="T13" s="19"/>
+      <c r="U13" s="19"/>
+      <c r="V13" s="19"/>
+      <c r="W13" s="19"/>
+      <c r="X13" s="19"/>
+      <c r="Y13" s="19"/>
     </row>
     <row r="14" spans="1:25" ht="43.95" customHeight="1">
-      <c r="A14" s="39"/>
-      <c r="B14" s="36"/>
-      <c r="C14" s="36"/>
-      <c r="D14" s="36"/>
-      <c r="E14" s="36"/>
-      <c r="F14" s="36"/>
-      <c r="G14" s="36"/>
-      <c r="H14" s="37" t="s">
+      <c r="A14" s="27"/>
+      <c r="B14" s="19"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="19"/>
+      <c r="H14" s="20" t="s">
         <v>98</v>
       </c>
-      <c r="I14" s="36"/>
-      <c r="J14" s="36"/>
-      <c r="K14" s="36"/>
-      <c r="L14" s="36"/>
-      <c r="M14" s="36"/>
-      <c r="N14" s="36"/>
-      <c r="O14" s="36"/>
-      <c r="P14" s="36"/>
-      <c r="Q14" s="36"/>
-      <c r="R14" s="36"/>
-      <c r="S14" s="36"/>
-      <c r="T14" s="36"/>
-      <c r="U14" s="36"/>
-      <c r="V14" s="36"/>
-      <c r="W14" s="36"/>
-      <c r="X14" s="36"/>
-      <c r="Y14" s="36"/>
+      <c r="I14" s="19"/>
+      <c r="J14" s="19"/>
+      <c r="K14" s="19"/>
+      <c r="L14" s="19"/>
+      <c r="M14" s="19"/>
+      <c r="N14" s="19"/>
+      <c r="O14" s="19"/>
+      <c r="P14" s="19"/>
+      <c r="Q14" s="19"/>
+      <c r="R14" s="19"/>
+      <c r="S14" s="19"/>
+      <c r="T14" s="19"/>
+      <c r="U14" s="19"/>
+      <c r="V14" s="19"/>
+      <c r="W14" s="19"/>
+      <c r="X14" s="19"/>
+      <c r="Y14" s="19"/>
     </row>
     <row r="15" spans="1:25" ht="43.95" customHeight="1">
-      <c r="A15" s="40"/>
-      <c r="B15" s="36"/>
-      <c r="C15" s="36"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="36"/>
-      <c r="F15" s="36"/>
-      <c r="G15" s="36"/>
-      <c r="H15" s="36"/>
-      <c r="I15" s="36"/>
-      <c r="J15" s="36"/>
-      <c r="K15" s="36"/>
-      <c r="L15" s="36"/>
-      <c r="M15" s="36"/>
-      <c r="N15" s="36"/>
-      <c r="O15" s="36"/>
-      <c r="P15" s="36"/>
-      <c r="Q15" s="36"/>
-      <c r="R15" s="36"/>
-      <c r="S15" s="36"/>
-      <c r="T15" s="36"/>
-      <c r="U15" s="36"/>
-      <c r="V15" s="36"/>
-      <c r="W15" s="36"/>
-      <c r="X15" s="36"/>
-      <c r="Y15" s="36"/>
+      <c r="A15" s="28"/>
+      <c r="B15" s="19"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
+      <c r="G15" s="19"/>
+      <c r="H15" s="19"/>
+      <c r="I15" s="19"/>
+      <c r="J15" s="19"/>
+      <c r="K15" s="19"/>
+      <c r="L15" s="19"/>
+      <c r="M15" s="19"/>
+      <c r="N15" s="19"/>
+      <c r="O15" s="19"/>
+      <c r="P15" s="19"/>
+      <c r="Q15" s="19"/>
+      <c r="R15" s="19"/>
+      <c r="S15" s="19"/>
+      <c r="T15" s="19"/>
+      <c r="U15" s="19"/>
+      <c r="V15" s="19"/>
+      <c r="W15" s="19"/>
+      <c r="X15" s="19"/>
+      <c r="Y15" s="19"/>
     </row>
     <row r="16" spans="1:25" ht="16.05" customHeight="1">
-      <c r="A16" s="27" t="s">
+      <c r="A16" s="42" t="s">
         <v>66</v>
       </c>
-      <c r="B16" s="26" t="s">
+      <c r="B16" s="41" t="s">
         <v>84</v>
       </c>
-      <c r="C16" s="20"/>
-      <c r="D16" s="20"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="20"/>
-      <c r="H16" s="20"/>
-      <c r="I16" s="20"/>
-      <c r="J16" s="20"/>
-      <c r="K16" s="20"/>
-      <c r="L16" s="20"/>
-      <c r="M16" s="20"/>
-      <c r="N16" s="20"/>
-      <c r="O16" s="20"/>
-      <c r="P16" s="20"/>
-      <c r="Q16" s="20"/>
-      <c r="R16" s="20"/>
-      <c r="S16" s="20"/>
-      <c r="T16" s="20"/>
-      <c r="U16" s="20"/>
-      <c r="V16" s="20"/>
-      <c r="W16" s="20"/>
-      <c r="X16" s="20"/>
-      <c r="Y16" s="20"/>
-    </row>
-    <row r="17" spans="1:25" ht="43.95" customHeight="1">
-      <c r="A17" s="22"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
+      <c r="I16" s="24"/>
+      <c r="J16" s="24"/>
+      <c r="K16" s="24"/>
+      <c r="L16" s="24"/>
+      <c r="M16" s="24"/>
+      <c r="N16" s="24"/>
+      <c r="O16" s="24"/>
+      <c r="P16" s="24"/>
+      <c r="Q16" s="24"/>
+      <c r="R16" s="24"/>
+      <c r="S16" s="24"/>
+      <c r="T16" s="24"/>
+      <c r="U16" s="24"/>
+      <c r="V16" s="24"/>
+      <c r="W16" s="24"/>
+      <c r="X16" s="24"/>
+      <c r="Y16" s="24"/>
+    </row>
+    <row r="17" spans="1:25" ht="127.2" customHeight="1">
+      <c r="A17" s="30"/>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
       <c r="D17" s="7"/>
@@ -1706,21 +1745,35 @@
       <c r="K17" s="7"/>
       <c r="L17" s="7"/>
       <c r="M17" s="7"/>
-      <c r="N17" s="7"/>
-      <c r="O17" s="7"/>
-      <c r="P17" s="7"/>
-      <c r="Q17" s="7"/>
-      <c r="R17" s="7"/>
-      <c r="S17" s="7"/>
-      <c r="T17" s="7"/>
+      <c r="N17" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="O17" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="P17" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="Q17" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="R17" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="S17" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="T17" s="7" t="s">
+        <v>110</v>
+      </c>
       <c r="U17" s="7"/>
       <c r="V17" s="7"/>
       <c r="W17" s="7"/>
       <c r="X17" s="7"/>
       <c r="Y17" s="7"/>
     </row>
-    <row r="18" spans="1:25" ht="43.95" customHeight="1">
-      <c r="A18" s="22"/>
+    <row r="18" spans="1:25" ht="134.4" customHeight="1">
+      <c r="A18" s="30"/>
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
       <c r="D18" s="7"/>
@@ -1733,21 +1786,33 @@
       <c r="K18" s="7"/>
       <c r="L18" s="7"/>
       <c r="M18" s="7"/>
-      <c r="N18" s="7"/>
+      <c r="N18" s="7" t="s">
+        <v>100</v>
+      </c>
       <c r="O18" s="7"/>
-      <c r="P18" s="7"/>
-      <c r="Q18" s="7"/>
-      <c r="R18" s="7"/>
-      <c r="S18" s="7"/>
-      <c r="T18" s="7"/>
+      <c r="P18" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="Q18" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="R18" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="S18" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="T18" s="7" t="s">
+        <v>111</v>
+      </c>
       <c r="U18" s="7"/>
       <c r="V18" s="7"/>
       <c r="W18" s="7"/>
       <c r="X18" s="7"/>
       <c r="Y18" s="7"/>
     </row>
-    <row r="19" spans="1:25" ht="43.95" customHeight="1">
-      <c r="A19" s="22"/>
+    <row r="19" spans="1:25" ht="138" customHeight="1">
+      <c r="A19" s="30"/>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
       <c r="D19" s="7"/>
@@ -1760,7 +1825,9 @@
       <c r="K19" s="7"/>
       <c r="L19" s="7"/>
       <c r="M19" s="7"/>
-      <c r="N19" s="7"/>
+      <c r="N19" s="7" t="s">
+        <v>101</v>
+      </c>
       <c r="O19" s="7"/>
       <c r="P19" s="7"/>
       <c r="Q19" s="7"/>
@@ -1774,7 +1841,7 @@
       <c r="Y19" s="7"/>
     </row>
     <row r="20" spans="1:25" ht="43.95" customHeight="1">
-      <c r="A20" s="23"/>
+      <c r="A20" s="31"/>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
       <c r="D20" s="7"/>
@@ -1801,38 +1868,38 @@
       <c r="Y20" s="7"/>
     </row>
     <row r="21" spans="1:25" ht="16.05" customHeight="1">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="38" t="s">
         <v>66</v>
       </c>
-      <c r="B21" s="19" t="s">
+      <c r="B21" s="37" t="s">
         <v>85</v>
       </c>
-      <c r="C21" s="20"/>
-      <c r="D21" s="20"/>
-      <c r="E21" s="20"/>
-      <c r="F21" s="20"/>
-      <c r="G21" s="20"/>
-      <c r="H21" s="20"/>
-      <c r="I21" s="20"/>
-      <c r="J21" s="20"/>
-      <c r="K21" s="20"/>
-      <c r="L21" s="20"/>
-      <c r="M21" s="20"/>
-      <c r="N21" s="20"/>
-      <c r="O21" s="20"/>
-      <c r="P21" s="20"/>
-      <c r="Q21" s="20"/>
-      <c r="R21" s="20"/>
-      <c r="S21" s="20"/>
-      <c r="T21" s="20"/>
-      <c r="U21" s="20"/>
-      <c r="V21" s="20"/>
-      <c r="W21" s="20"/>
-      <c r="X21" s="20"/>
-      <c r="Y21" s="20"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="24"/>
+      <c r="G21" s="24"/>
+      <c r="H21" s="24"/>
+      <c r="I21" s="24"/>
+      <c r="J21" s="24"/>
+      <c r="K21" s="24"/>
+      <c r="L21" s="24"/>
+      <c r="M21" s="24"/>
+      <c r="N21" s="24"/>
+      <c r="O21" s="24"/>
+      <c r="P21" s="24"/>
+      <c r="Q21" s="24"/>
+      <c r="R21" s="24"/>
+      <c r="S21" s="24"/>
+      <c r="T21" s="24"/>
+      <c r="U21" s="24"/>
+      <c r="V21" s="24"/>
+      <c r="W21" s="24"/>
+      <c r="X21" s="24"/>
+      <c r="Y21" s="24"/>
     </row>
     <row r="22" spans="1:25" ht="43.95" customHeight="1">
-      <c r="A22" s="22"/>
+      <c r="A22" s="30"/>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
       <c r="D22" s="8"/>
@@ -1859,7 +1926,7 @@
       <c r="Y22" s="8"/>
     </row>
     <row r="23" spans="1:25" ht="43.95" customHeight="1">
-      <c r="A23" s="22"/>
+      <c r="A23" s="30"/>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
       <c r="D23" s="8"/>
@@ -1886,7 +1953,7 @@
       <c r="Y23" s="8"/>
     </row>
     <row r="24" spans="1:25" ht="43.95" customHeight="1">
-      <c r="A24" s="22"/>
+      <c r="A24" s="30"/>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
       <c r="D24" s="8"/>
@@ -1913,7 +1980,7 @@
       <c r="Y24" s="8"/>
     </row>
     <row r="25" spans="1:25" ht="43.95" customHeight="1">
-      <c r="A25" s="23"/>
+      <c r="A25" s="31"/>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
       <c r="D25" s="8"/>
@@ -1941,6 +2008,14 @@
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="B21:Y21"/>
+    <mergeCell ref="A21:A25"/>
+    <mergeCell ref="Q3:R3"/>
+    <mergeCell ref="M3:P3"/>
+    <mergeCell ref="B11:Y11"/>
+    <mergeCell ref="S3:T3"/>
+    <mergeCell ref="B16:Y16"/>
+    <mergeCell ref="A16:A20"/>
     <mergeCell ref="A1:Y1"/>
     <mergeCell ref="M2:P2"/>
     <mergeCell ref="A11:A15"/>
@@ -1956,14 +2031,6 @@
     <mergeCell ref="B6:Y6"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="U3:Y3"/>
-    <mergeCell ref="B21:Y21"/>
-    <mergeCell ref="A21:A25"/>
-    <mergeCell ref="Q3:R3"/>
-    <mergeCell ref="M3:P3"/>
-    <mergeCell ref="B11:Y11"/>
-    <mergeCell ref="S3:T3"/>
-    <mergeCell ref="B16:Y16"/>
-    <mergeCell ref="A16:A20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>